<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-18 19:26 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -2456,7 +2456,7 @@
         <v>46128.431861122684</v>
       </c>
       <c r="D19" s="8">
-        <v>46128.4318752199</v>
+        <v>46191.801118738425</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>80</v>
@@ -2765,11 +2765,9 @@
       <c r="B24" s="5">
         <v>46079.83530122685</v>
       </c>
-      <c r="C24" s="5">
-        <v>46114.765597731486</v>
-      </c>
+      <c r="C24" s="6"/>
       <c r="D24" s="5">
-        <v>46114.765615625</v>
+        <v>46191.80108803241</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>97</v>
@@ -2831,10 +2829,10 @@
         <v>46079.87430951389</v>
       </c>
       <c r="C25" s="8">
-        <v>46114.515038530095</v>
+        <v>46191.80111393519</v>
       </c>
       <c r="D25" s="8">
-        <v>46114.51506849537</v>
+        <v>46191.801115636576</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>102</v>
@@ -2896,10 +2894,10 @@
         <v>46080.51039956018</v>
       </c>
       <c r="C26" s="5">
-        <v>46114.515089340275</v>
+        <v>46191.801125949074</v>
       </c>
       <c r="D26" s="5">
-        <v>46158.995789374996</v>
+        <v>46191.80112726852</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>105</v>
@@ -2962,7 +2960,7 @@
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="8">
-        <v>46158.992551006944</v>
+        <v>46191.801205324075</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>107</v>
@@ -3798,11 +3796,9 @@
       <c r="B41" s="8">
         <v>46079.835302418986</v>
       </c>
-      <c r="C41" s="8">
-        <v>46114.765703530094</v>
-      </c>
+      <c r="C41" s="9"/>
       <c r="D41" s="8">
-        <v>46147.193391990746</v>
+        <v>46191.801202013885</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>152</v>
@@ -3867,7 +3863,7 @@
         <v>46114.765637812496</v>
       </c>
       <c r="D42" s="5">
-        <v>46114.765639097226</v>
+        <v>46191.80109314815</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>157</v>
@@ -4054,7 +4050,7 @@
         <v>46114.7660537037</v>
       </c>
       <c r="D45" s="8">
-        <v>46114.766054872685</v>
+        <v>46191.80111972222</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>166</v>
@@ -4479,11 +4475,9 @@
       <c r="B52" s="5">
         <v>46079.835301053245</v>
       </c>
-      <c r="C52" s="5">
-        <v>46191.79630699074</v>
-      </c>
+      <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46191.79631972223</v>
+        <v>46191.80128876158</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>192</v>
@@ -4534,11 +4528,9 @@
       <c r="B53" s="8">
         <v>46079.835301342595</v>
       </c>
-      <c r="C53" s="8">
-        <v>46191.79629</v>
-      </c>
+      <c r="C53" s="9"/>
       <c r="D53" s="8">
-        <v>46191.79630796296</v>
+        <v>46191.80125251158</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>195</v>
@@ -4599,11 +4591,9 @@
       <c r="B54" s="5">
         <v>46079.83530162037</v>
       </c>
-      <c r="C54" s="5">
-        <v>46191.79562175926</v>
-      </c>
+      <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46191.7963069213</v>
+        <v>46191.80126277778</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>200</v>
@@ -4719,7 +4709,7 @@
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46191.795639421296</v>
+        <v>46191.80126917824</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>206</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-01 21:54 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -269,6 +269,9 @@
     <t>propuesta motor,propuesta alabes,propuesta nucleo rodete,propuesta tableros,propuesta compras a codigo // aprovisionamiento,Propuesta Sensores</t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
     <t>1213459189153321</t>
   </si>
   <si>
@@ -276,9 +279,6 @@
   </si>
   <si>
     <t>Propuesta compras:,Generación OC Alabe ot 4264</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1213459189153322</t>
@@ -2456,7 +2456,7 @@
         <v>46128.431861122684</v>
       </c>
       <c r="D19" s="8">
-        <v>46191.801118738425</v>
+        <v>46204.90569222222</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>80</v>
@@ -2493,14 +2493,14 @@
       <c r="S19" s="9">
         <v>1</v>
       </c>
-      <c r="T19" s="10" t="s">
-        <v>31</v>
+      <c r="T19" s="12" t="s">
+        <v>82</v>
       </c>
       <c r="U19" s="9"/>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B20" s="5">
         <v>46079.83530313657</v>
@@ -2512,7 +2512,7 @@
         <v>46111.79283396991</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
@@ -2545,7 +2545,7 @@
         <v>67</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="Q20" s="5">
         <v>46093</v>
@@ -2557,7 +2557,7 @@
         <v>1</v>
       </c>
       <c r="T20" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="U20" s="11" t="s">
         <v>32</v>
@@ -2765,9 +2765,11 @@
       <c r="B24" s="5">
         <v>46079.83530122685</v>
       </c>
-      <c r="C24" s="6"/>
+      <c r="C24" s="5">
+        <v>46204.90566989583</v>
+      </c>
       <c r="D24" s="5">
-        <v>46196.639933819446</v>
+        <v>46204.90567366898</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>97</v>
@@ -2996,7 +2998,7 @@
       <c r="R27" s="9"/>
       <c r="S27" s="9"/>
       <c r="T27" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="U27" s="9"/>
     </row>
@@ -3109,7 +3111,7 @@
         <v>110</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="P29" s="9" t="s">
         <v>116</v>
@@ -3433,7 +3435,7 @@
         <v>1</v>
       </c>
       <c r="T34" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="U34" s="11" t="s">
         <v>32</v>
@@ -3885,7 +3887,7 @@
         <v>46114.765637812496</v>
       </c>
       <c r="D42" s="5">
-        <v>46191.80109314815</v>
+        <v>46204.90568498842</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>157</v>
@@ -4663,7 +4665,7 @@
         <v>1</v>
       </c>
       <c r="T54" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="U54" s="11" t="s">
         <v>32</v>
@@ -4779,7 +4781,7 @@
         <v>0</v>
       </c>
       <c r="T56" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="U56" s="11" t="s">
         <v>32</v>
@@ -5021,7 +5023,7 @@
         <v>0</v>
       </c>
       <c r="T60" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="U60" s="10" t="s">
         <v>117</v>
@@ -5084,7 +5086,7 @@
         <v>0</v>
       </c>
       <c r="T61" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="U61" s="11" t="s">
         <v>32</v>
@@ -5147,7 +5149,7 @@
         <v>0</v>
       </c>
       <c r="T62" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="U62" s="12" t="s">
         <v>59</v>
@@ -5210,7 +5212,7 @@
         <v>0</v>
       </c>
       <c r="T63" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="U63" s="11" t="s">
         <v>32</v>
@@ -5273,7 +5275,7 @@
         <v>0</v>
       </c>
       <c r="T64" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="U64" s="10" t="s">
         <v>117</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-05 01:25 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -200,169 +200,169 @@
     <t>Tarea sin iniciar</t>
   </si>
   <si>
+    <t>1213459189153314</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:</t>
+  </si>
+  <si>
+    <t>Ingenieria basica Damper,Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete,Analisis de costeo</t>
+  </si>
+  <si>
+    <t>1213459189153315</t>
+  </si>
+  <si>
+    <t>Ingenieria Basica Motor</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
+  </si>
+  <si>
+    <t>1213459189153317</t>
+  </si>
+  <si>
+    <t>Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta nucleo rodete,propuesta alabes</t>
+  </si>
+  <si>
+    <t>1213459189153318</t>
+  </si>
+  <si>
+    <t>Ingenieria Detalle</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta compras a codigo // aprovisionamiento,Propuesta Sensores,Planos preliminar</t>
+  </si>
+  <si>
+    <t>1213458011369803</t>
+  </si>
+  <si>
+    <t>Ingenieria basica Damper</t>
+  </si>
+  <si>
+    <t>Analisis de costeo,Propuesta Damper,Ingenieria Jefe de proyecto:</t>
+  </si>
+  <si>
+    <t>1213459189153319</t>
+  </si>
+  <si>
+    <t>Analisis de costeo</t>
+  </si>
+  <si>
+    <t>Ingenieria basica Damper,Ingenieria Basica Motor,Ingenieria Detalle,Ingenieria basica Rodete</t>
+  </si>
+  <si>
+    <t>Ingenieria Jefe de proyecto:,Costos</t>
+  </si>
+  <si>
+    <t>1213459189153320</t>
+  </si>
+  <si>
+    <t>Propuesta compras:</t>
+  </si>
+  <si>
+    <t>propuesta motor,propuesta alabes,propuesta nucleo rodete,propuesta tableros,propuesta compras a codigo // aprovisionamiento,Propuesta Sensores</t>
+  </si>
+  <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
+    <t>1213459189153321</t>
+  </si>
+  <si>
+    <t>propuesta alabes</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Alabe ot 4264</t>
+  </si>
+  <si>
+    <t>1213459189153322</t>
+  </si>
+  <si>
+    <t>propuesta motor</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC motor ot 4264</t>
+  </si>
+  <si>
+    <t>1213459189153323</t>
+  </si>
+  <si>
+    <t>propuesta tableros</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Tableros  ot 4265 - ot 4266</t>
+  </si>
+  <si>
+    <t>1213459189153324</t>
+  </si>
+  <si>
+    <t>propuesta nucleo rodete</t>
+  </si>
+  <si>
+    <t>benjamin.bustos@zitron.com</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Rodete ot 4264</t>
+  </si>
+  <si>
+    <t>1213459189153325</t>
+  </si>
+  <si>
+    <t>propuesta compras a codigo // aprovisionamiento</t>
+  </si>
+  <si>
+    <t>hugo isla martinez</t>
+  </si>
+  <si>
+    <t>hugo.isla@zitron.com</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC materiales</t>
+  </si>
+  <si>
+    <t>1213458788103036</t>
+  </si>
+  <si>
+    <t>Propuesta Sensores</t>
+  </si>
+  <si>
+    <t>Propuesta compras:,Generación OC Sensores</t>
+  </si>
+  <si>
+    <t>1213458011369804</t>
+  </si>
+  <si>
+    <t>Propuesta Damper</t>
+  </si>
+  <si>
+    <t>1213459189153326</t>
+  </si>
+  <si>
+    <t>Compras:</t>
+  </si>
+  <si>
+    <t>Sensores,Materiales a codigo // compras locales aprovisionamientomiento:,rodete ot 4264,Tablero ot 4265 - ot 4266,Motor ot 4264,Alabe  ot 4264</t>
+  </si>
+  <si>
+    <t>1213459189153327</t>
+  </si>
+  <si>
+    <t>Alabe  ot 4264</t>
+  </si>
+  <si>
+    <t>Eliana</t>
+  </si>
+  <si>
+    <t>ecarico@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe ot 4264,Fabricación Alabe ot 4264</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213459189153314</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:</t>
-  </si>
-  <si>
-    <t>Ingenieria basica Damper,Ingenieria Detalle,Ingenieria Basica Motor,Ingenieria basica Rodete,Analisis de costeo</t>
-  </si>
-  <si>
-    <t>1213459189153315</t>
-  </si>
-  <si>
-    <t>Ingenieria Basica Motor</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta motor</t>
-  </si>
-  <si>
-    <t>1213459189153317</t>
-  </si>
-  <si>
-    <t>Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta nucleo rodete,propuesta alabes</t>
-  </si>
-  <si>
-    <t>1213459189153318</t>
-  </si>
-  <si>
-    <t>Ingenieria Detalle</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Ingenieria Jefe de proyecto:,propuesta compras a codigo // aprovisionamiento,Propuesta Sensores,Planos preliminar</t>
-  </si>
-  <si>
-    <t>1213458011369803</t>
-  </si>
-  <si>
-    <t>Ingenieria basica Damper</t>
-  </si>
-  <si>
-    <t>Analisis de costeo,Propuesta Damper,Ingenieria Jefe de proyecto:</t>
-  </si>
-  <si>
-    <t>1213459189153319</t>
-  </si>
-  <si>
-    <t>Analisis de costeo</t>
-  </si>
-  <si>
-    <t>Ingenieria basica Damper,Ingenieria Basica Motor,Ingenieria Detalle,Ingenieria basica Rodete</t>
-  </si>
-  <si>
-    <t>Ingenieria Jefe de proyecto:,Costos</t>
-  </si>
-  <si>
-    <t>1213459189153320</t>
-  </si>
-  <si>
-    <t>Propuesta compras:</t>
-  </si>
-  <si>
-    <t>propuesta motor,propuesta alabes,propuesta nucleo rodete,propuesta tableros,propuesta compras a codigo // aprovisionamiento,Propuesta Sensores</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1213459189153321</t>
-  </si>
-  <si>
-    <t>propuesta alabes</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Alabe ot 4264</t>
-  </si>
-  <si>
-    <t>1213459189153322</t>
-  </si>
-  <si>
-    <t>propuesta motor</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC motor ot 4264</t>
-  </si>
-  <si>
-    <t>1213459189153323</t>
-  </si>
-  <si>
-    <t>propuesta tableros</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Tableros  ot 4265 - ot 4266</t>
-  </si>
-  <si>
-    <t>1213459189153324</t>
-  </si>
-  <si>
-    <t>propuesta nucleo rodete</t>
-  </si>
-  <si>
-    <t>benjamin.bustos@zitron.com</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Rodete ot 4264</t>
-  </si>
-  <si>
-    <t>1213459189153325</t>
-  </si>
-  <si>
-    <t>propuesta compras a codigo // aprovisionamiento</t>
-  </si>
-  <si>
-    <t>hugo isla martinez</t>
-  </si>
-  <si>
-    <t>hugo.isla@zitron.com</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC materiales</t>
-  </si>
-  <si>
-    <t>1213458788103036</t>
-  </si>
-  <si>
-    <t>Propuesta Sensores</t>
-  </si>
-  <si>
-    <t>Propuesta compras:,Generación OC Sensores</t>
-  </si>
-  <si>
-    <t>1213458011369804</t>
-  </si>
-  <si>
-    <t>Propuesta Damper</t>
-  </si>
-  <si>
-    <t>1213459189153326</t>
-  </si>
-  <si>
-    <t>Compras:</t>
-  </si>
-  <si>
-    <t>Sensores,Materiales a codigo // compras locales aprovisionamientomiento:,rodete ot 4264,Tablero ot 4265 - ot 4266,Motor ot 4264,Alabe  ot 4264</t>
-  </si>
-  <si>
-    <t>1213459189153327</t>
-  </si>
-  <si>
-    <t>Alabe  ot 4264</t>
-  </si>
-  <si>
-    <t>Eliana</t>
-  </si>
-  <si>
-    <t>ecarico@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe ot 4264,Fabricación Alabe ot 4264</t>
   </si>
   <si>
     <t>1213459189153328</t>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46206.25029707176</v>
+        <v>46207.20142103009</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>55</v>
@@ -2063,13 +2063,13 @@
       <c r="T12" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="U12" s="12" t="s">
-        <v>59</v>
+      <c r="U12" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="8">
         <v>46079.83530335648</v>
@@ -2081,7 +2081,7 @@
         <v>46114.51491809028</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>25</v>
@@ -2105,7 +2105,7 @@
         <v>26</v>
       </c>
       <c r="O13" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P13" s="9" t="s">
         <v>26</v>
@@ -2122,7 +2122,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B14" s="5">
         <v>46079.83530126157</v>
@@ -2134,7 +2134,7 @@
         <v>46114.5143725</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>26</v>
@@ -2161,13 +2161,13 @@
         <v>26</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>40</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="Q14" s="5">
         <v>46084</v>
@@ -2187,7 +2187,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B15" s="8">
         <v>46079.83530193287</v>
@@ -2199,7 +2199,7 @@
         <v>46111.79282915509</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>26</v>
@@ -2226,13 +2226,13 @@
         <v>26</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>40</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Q15" s="8">
         <v>46084</v>
@@ -2252,7 +2252,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B16" s="5">
         <v>46079.83530225694</v>
@@ -2264,7 +2264,7 @@
         <v>46114.51447722223</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
@@ -2291,13 +2291,13 @@
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>40</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="Q16" s="5">
         <v>46084</v>
@@ -2317,7 +2317,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B17" s="8">
         <v>46080.51025131944</v>
@@ -2329,7 +2329,7 @@
         <v>46114.51483395833</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>26</v>
@@ -2356,13 +2356,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O17" s="9" t="s">
         <v>40</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Q17" s="8">
         <v>46084</v>
@@ -2382,7 +2382,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B18" s="5">
         <v>46079.83530255787</v>
@@ -2394,7 +2394,7 @@
         <v>46114.51490420139</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>26</v>
@@ -2421,13 +2421,13 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="O18" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="P18" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="P18" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="Q18" s="5">
         <v>46084</v>
@@ -2447,7 +2447,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B19" s="8">
         <v>46079.83530284722</v>
@@ -2459,7 +2459,7 @@
         <v>46204.90569222222</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>25</v>
@@ -2483,7 +2483,7 @@
         <v>26</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="P19" s="9" t="s">
         <v>26</v>
@@ -2494,13 +2494,13 @@
         <v>1</v>
       </c>
       <c r="T19" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U19" s="9"/>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B20" s="5">
         <v>46079.83530313657</v>
@@ -2512,7 +2512,7 @@
         <v>46111.79283396991</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
@@ -2539,13 +2539,13 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="Q20" s="5">
         <v>46093</v>
@@ -2557,7 +2557,7 @@
         <v>1</v>
       </c>
       <c r="T20" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U20" s="11" t="s">
         <v>32</v>
@@ -2565,7 +2565,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B21" s="8">
         <v>46079.8353034375</v>
@@ -2577,7 +2577,7 @@
         <v>46114.514961354165</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>26</v>
@@ -2604,13 +2604,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O21" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Q21" s="8">
         <v>46086</v>
@@ -2630,7 +2630,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B22" s="5">
         <v>46079.83530375</v>
@@ -2642,7 +2642,7 @@
         <v>46142.66126559028</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>26</v>
@@ -2669,13 +2669,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O22" s="6" t="s">
         <v>49</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="Q22" s="5">
         <v>46087</v>
@@ -2695,7 +2695,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B23" s="8">
         <v>46079.835304050925</v>
@@ -2707,16 +2707,16 @@
         <v>46129.00161702547</v>
       </c>
       <c r="E23" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G23" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="F23" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>94</v>
-      </c>
       <c r="H23" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I23" s="8">
         <v>46093</v>
@@ -2734,13 +2734,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="Q23" s="8">
         <v>46093</v>
@@ -2760,7 +2760,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B24" s="5">
         <v>46079.83530122685</v>
@@ -2772,16 +2772,16 @@
         <v>46204.90567366898</v>
       </c>
       <c r="E24" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="F24" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G24" s="6" t="s">
+      <c r="H24" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>99</v>
       </c>
       <c r="I24" s="5">
         <v>46093</v>
@@ -2799,13 +2799,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q24" s="5">
         <v>46093</v>
@@ -2825,7 +2825,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B25" s="8">
         <v>46079.87430951389</v>
@@ -2837,7 +2837,7 @@
         <v>46191.801115636576</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>26</v>
@@ -2864,13 +2864,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="P25" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="Q25" s="8">
         <v>46093</v>
@@ -2890,7 +2890,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B26" s="5">
         <v>46080.51039956018</v>
@@ -2902,7 +2902,7 @@
         <v>46191.80112726852</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
@@ -2929,10 +2929,10 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>26</v>
@@ -2955,7 +2955,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B27" s="8">
         <v>46079.83530158565</v>
@@ -2965,7 +2965,7 @@
         <v>46191.87501525463</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>25</v>
@@ -2989,7 +2989,7 @@
         <v>26</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="P27" s="9" t="s">
         <v>26</v>
@@ -2998,13 +2998,13 @@
       <c r="R27" s="9"/>
       <c r="S27" s="9"/>
       <c r="T27" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U27" s="9"/>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B28" s="5">
         <v>46079.83530186342</v>
@@ -3016,16 +3016,16 @@
         <v>46204.193195381944</v>
       </c>
       <c r="E28" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G28" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="F28" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G28" s="6" t="s">
+      <c r="H28" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="I28" s="5">
         <v>46097</v>
@@ -3043,13 +3043,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q28" s="5">
         <v>46097</v>
@@ -3064,7 +3064,7 @@
         <v>31</v>
       </c>
       <c r="U28" s="12" t="s">
-        <v>59</v>
+        <v>113</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3087,10 +3087,10 @@
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H29" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="H29" s="9" t="s">
-        <v>112</v>
       </c>
       <c r="I29" s="8">
         <v>46097</v>
@@ -3108,10 +3108,10 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="P29" s="9" t="s">
         <v>116</v>
@@ -3148,10 +3148,10 @@
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="H30" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="I30" s="5">
         <v>46099</v>
@@ -3169,7 +3169,7 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O30" s="6" t="s">
         <v>115</v>
@@ -3209,10 +3209,10 @@
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="H31" s="9" t="s">
-        <v>112</v>
       </c>
       <c r="I31" s="8">
         <v>46091</v>
@@ -3230,13 +3230,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O31" s="9" t="s">
         <v>123</v>
       </c>
       <c r="P31" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q31" s="8">
         <v>46091</v>
@@ -3274,10 +3274,10 @@
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="I32" s="5">
         <v>46091</v>
@@ -3298,7 +3298,7 @@
         <v>122</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P32" s="6" t="s">
         <v>126</v>
@@ -3335,10 +3335,10 @@
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H33" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="H33" s="9" t="s">
-        <v>112</v>
       </c>
       <c r="I33" s="8">
         <v>46100</v>
@@ -3396,10 +3396,10 @@
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="I34" s="5">
         <v>46090</v>
@@ -3417,13 +3417,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>132</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q34" s="5">
         <v>46090</v>
@@ -3435,7 +3435,7 @@
         <v>1</v>
       </c>
       <c r="T34" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U34" s="11" t="s">
         <v>32</v>
@@ -3461,10 +3461,10 @@
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H35" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="H35" s="9" t="s">
-        <v>112</v>
       </c>
       <c r="I35" s="8">
         <v>46090</v>
@@ -3485,7 +3485,7 @@
         <v>131</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P35" s="9" t="s">
         <v>135</v>
@@ -3522,10 +3522,10 @@
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="I36" s="5">
         <v>46108</v>
@@ -3583,10 +3583,10 @@
         <v>26</v>
       </c>
       <c r="G37" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H37" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>112</v>
       </c>
       <c r="I37" s="8">
         <v>46108</v>
@@ -3644,10 +3644,10 @@
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="H38" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="I38" s="5">
         <v>46097</v>
@@ -3665,13 +3665,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O38" s="6" t="s">
         <v>144</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q38" s="5">
         <v>46097</v>
@@ -3709,10 +3709,10 @@
         <v>26</v>
       </c>
       <c r="G39" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H39" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>112</v>
       </c>
       <c r="I39" s="8">
         <v>46097</v>
@@ -3733,7 +3733,7 @@
         <v>143</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="P39" s="9" t="s">
         <v>147</v>
@@ -3770,10 +3770,10 @@
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="I40" s="5">
         <v>46099</v>
@@ -3852,13 +3852,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O41" s="9" t="s">
         <v>155</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q41" s="8">
         <v>46097</v>
@@ -3920,7 +3920,7 @@
         <v>152</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>158</v>
@@ -4039,13 +4039,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>164</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="Q44" s="5">
         <v>46097</v>
@@ -4107,7 +4107,7 @@
         <v>163</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P45" s="9" t="s">
         <v>167</v>
@@ -4278,7 +4278,7 @@
         <v>172</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="P48" s="6" t="s">
         <v>178</v>
@@ -4665,7 +4665,7 @@
         <v>1</v>
       </c>
       <c r="T54" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U54" s="11" t="s">
         <v>32</v>
@@ -4781,7 +4781,7 @@
         <v>0</v>
       </c>
       <c r="T56" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U56" s="11" t="s">
         <v>32</v>
@@ -5023,10 +5023,10 @@
         <v>0</v>
       </c>
       <c r="T60" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U60" s="12" t="s">
-        <v>59</v>
+        <v>113</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -5086,7 +5086,7 @@
         <v>0</v>
       </c>
       <c r="T61" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U61" s="11" t="s">
         <v>32</v>
@@ -5149,7 +5149,7 @@
         <v>0</v>
       </c>
       <c r="T62" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U62" s="11" t="s">
         <v>32</v>
@@ -5212,7 +5212,7 @@
         <v>0</v>
       </c>
       <c r="T63" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U63" s="11" t="s">
         <v>32</v>
@@ -5275,7 +5275,7 @@
         <v>0</v>
       </c>
       <c r="T64" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="U64" s="10" t="s">
         <v>117</v>
@@ -5352,10 +5352,10 @@
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I66" s="5">
         <v>46195</v>
@@ -5394,7 +5394,7 @@
         <v>58</v>
       </c>
       <c r="U66" s="12" t="s">
-        <v>59</v>
+        <v>113</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -5415,10 +5415,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I67" s="8">
         <v>46238</v>
@@ -5478,10 +5478,10 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I68" s="5">
         <v>46216</v>
@@ -5541,10 +5541,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I69" s="8">
         <v>46218</v>
@@ -5604,10 +5604,10 @@
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I70" s="5">
         <v>46220</v>
@@ -5667,10 +5667,10 @@
         <v>26</v>
       </c>
       <c r="G71" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H71" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I71" s="8">
         <v>46240</v>
@@ -5730,10 +5730,10 @@
         <v>26</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I72" s="5">
         <v>46244</v>
@@ -5901,10 +5901,10 @@
         <v>26</v>
       </c>
       <c r="G75" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H75" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I75" s="8">
         <v>46246</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-06 17:07 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -2960,9 +2960,11 @@
       <c r="B27" s="8">
         <v>46079.83530158565</v>
       </c>
-      <c r="C27" s="9"/>
+      <c r="C27" s="8">
+        <v>46209.70945200232</v>
+      </c>
       <c r="D27" s="8">
-        <v>46191.87501525463</v>
+        <v>46209.709468483794</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>106</v>
@@ -2996,9 +2998,11 @@
       </c>
       <c r="Q27" s="9"/>
       <c r="R27" s="9"/>
-      <c r="S27" s="9"/>
-      <c r="T27" s="12" t="s">
-        <v>81</v>
+      <c r="S27" s="9">
+        <v>1</v>
+      </c>
+      <c r="T27" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U27" s="9"/>
     </row>
@@ -4975,7 +4979,7 @@
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46206.20063146991</v>
+        <v>46209.7099818287</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>221</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-09 13:29 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -362,334 +362,334 @@
     <t>Generación OC Alabe ot 4264,Fabricación Alabe ot 4264</t>
   </si>
   <si>
+    <t>1213459189153328</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe ot 4264</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe ot 4264,Alabe  ot 4264</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>1213459189153329</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe ot 4264</t>
+  </si>
+  <si>
+    <t>Alabe  ot 4264,Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>1213459189153330</t>
+  </si>
+  <si>
+    <t>Tablero ot 4265 - ot 4266</t>
+  </si>
+  <si>
+    <t>Generación OC Tableros  ot 4265 - ot 4266,Fabricación Tablero  ot 4265 - ot 4266</t>
+  </si>
+  <si>
+    <t>1213459189153331</t>
+  </si>
+  <si>
+    <t>Generación OC Tableros  ot 4265 - ot 4266</t>
+  </si>
+  <si>
+    <t>Fabricación Tablero  ot 4265 - ot 4266,Tablero ot 4265 - ot 4266</t>
+  </si>
+  <si>
+    <t>1213459189153332</t>
+  </si>
+  <si>
+    <t>Fabricación Tablero  ot 4265 - ot 4266</t>
+  </si>
+  <si>
+    <t>Tablero ot 4265 - ot 4266,Recepcion Tableros</t>
+  </si>
+  <si>
+    <t>1213459189153336</t>
+  </si>
+  <si>
+    <t>Motor ot 4264</t>
+  </si>
+  <si>
+    <t>Generación OC motor ot 4264,Fabricación motor ot 4264,Planos motor proveedor ot 4264</t>
+  </si>
+  <si>
+    <t>1213459189207060</t>
+  </si>
+  <si>
+    <t>Generación OC motor ot 4264</t>
+  </si>
+  <si>
+    <t>Fabricación motor ot 4264,Motor ot 4264,Planos motor proveedor ot 4264</t>
+  </si>
+  <si>
+    <t>1213459189207061</t>
+  </si>
+  <si>
+    <t>Fabricación motor ot 4264</t>
+  </si>
+  <si>
+    <t>Motor ot 4264,Recepcion motor</t>
+  </si>
+  <si>
+    <t>1213459189207062</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor ot 4264</t>
+  </si>
+  <si>
+    <t>Motor ot 4264,Ingenieria y diseño:,Planos definitivos</t>
+  </si>
+  <si>
+    <t>1213459189153333</t>
+  </si>
+  <si>
+    <t>rodete ot 4264</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete ot 4264,Fabricación Rodete ot 4264</t>
+  </si>
+  <si>
+    <t>1213459189153334</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete ot 4264</t>
+  </si>
+  <si>
+    <t>Fabricación Rodete ot 4264,rodete ot 4264</t>
+  </si>
+  <si>
+    <t>1213459189153335</t>
+  </si>
+  <si>
+    <t>Fabricación Rodete ot 4264</t>
+  </si>
+  <si>
+    <t>rodete ot 4264,Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>1213459189207063</t>
+  </si>
+  <si>
+    <t>Materiales a codigo // compras locales aprovisionamientomiento:</t>
+  </si>
+  <si>
+    <t>Yerlia Ayleen Castillo Diaz</t>
+  </si>
+  <si>
+    <t>yerlia.castillo@zitron.com</t>
+  </si>
+  <si>
+    <t>Generación OC materiales,Fabricacion a codigo y compras locales</t>
+  </si>
+  <si>
+    <t>1213459189207064</t>
+  </si>
+  <si>
+    <t>Generación OC materiales</t>
+  </si>
+  <si>
+    <t>Fabricacion a codigo y compras locales,Materiales a codigo // compras locales aprovisionamientomiento:</t>
+  </si>
+  <si>
+    <t>1213459189207065</t>
+  </si>
+  <si>
+    <t>Fabricacion a codigo y compras locales</t>
+  </si>
+  <si>
+    <t>Materiales a codigo // compras locales aprovisionamientomiento:,Recepcion materiales a codigos // compras locales aprovisionamiento</t>
+  </si>
+  <si>
+    <t>1213458788103037</t>
+  </si>
+  <si>
+    <t>Sensores</t>
+  </si>
+  <si>
+    <t>Generación OC Sensores,Fabricacion Sensores</t>
+  </si>
+  <si>
+    <t>1213458788103039</t>
+  </si>
+  <si>
+    <t>Generación OC Sensores</t>
+  </si>
+  <si>
+    <t>Fabricacion Sensores,Sensores</t>
+  </si>
+  <si>
+    <t>1213458788103040</t>
+  </si>
+  <si>
+    <t>Fabricacion Sensores</t>
+  </si>
+  <si>
+    <t>Sensores,Recepcion Sensores</t>
+  </si>
+  <si>
+    <t>1213459189207066</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseño:</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor ot 4264,Planos preliminar,Check plano,Check pruebas FAT</t>
+  </si>
+  <si>
+    <t>1213459189207067</t>
+  </si>
+  <si>
+    <t>Planos preliminar</t>
+  </si>
+  <si>
+    <t>Hernan Roberto Gutierrez Barrientos</t>
+  </si>
+  <si>
+    <t>hgutierrez@zitron.com</t>
+  </si>
+  <si>
+    <t>Ingenieria y diseño:,Planos definitivos,Ingenieria Y diseño</t>
+  </si>
+  <si>
+    <t>1213459189207068</t>
+  </si>
+  <si>
+    <t>Planos definitivos</t>
+  </si>
+  <si>
+    <t>Francisca González Cornejo</t>
+  </si>
+  <si>
+    <t>francisca.gonzalez@zitron.com</t>
+  </si>
+  <si>
+    <t>Planos preliminar,Planos motor proveedor ot 4264</t>
+  </si>
+  <si>
+    <t>Check plano</t>
+  </si>
+  <si>
+    <t>1213560053852552</t>
+  </si>
+  <si>
+    <t>Armado,Control de calidad Armado,Ingenieria y diseño:,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje sensor</t>
+  </si>
+  <si>
+    <t>1213560053852553</t>
+  </si>
+  <si>
+    <t>Check pruebas FAT</t>
+  </si>
+  <si>
+    <t>Pruebas FAT</t>
+  </si>
+  <si>
+    <t>RE-PINTADO,Ingenieria y diseño:</t>
+  </si>
+  <si>
+    <t>1213459189207069</t>
+  </si>
+  <si>
+    <t>Bodega:</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Recepcion materiales a codigos // compras locales aprovisionamiento</t>
+  </si>
+  <si>
+    <t>1213459189207070</t>
+  </si>
+  <si>
+    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Victor Muñoz</t>
+  </si>
+  <si>
+    <t>victor.munoz@zitron.com</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Bodega:</t>
+  </si>
+  <si>
+    <t>1213459189207071</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Nicolás López</t>
+  </si>
+  <si>
+    <t>nicolas.lopez@zitron.com</t>
+  </si>
+  <si>
+    <t>Bodega:,Preparación Materiales</t>
+  </si>
+  <si>
+    <t>1213459189207072</t>
+  </si>
+  <si>
+    <t>Caldereria:</t>
+  </si>
+  <si>
+    <t>Preparación Materiales</t>
+  </si>
+  <si>
+    <t>1213459189207073</t>
+  </si>
+  <si>
+    <t>Nicolás Mol</t>
+  </si>
+  <si>
+    <t>nicolas.mol@zitron.com</t>
+  </si>
+  <si>
+    <t>Caldereria:,Armado,Armado</t>
+  </si>
+  <si>
+    <t>1213459189207074</t>
+  </si>
+  <si>
+    <t>Armado</t>
+  </si>
+  <si>
+    <t>Preparación Materiales,Check plano</t>
+  </si>
+  <si>
+    <t>Control de calidad Armado</t>
+  </si>
+  <si>
+    <t>1213459189207075</t>
+  </si>
+  <si>
+    <t>Armado,Check plano</t>
+  </si>
+  <si>
+    <t>Revestimiento</t>
+  </si>
+  <si>
+    <t>1213459189207076</t>
+  </si>
+  <si>
+    <t>Recepcion Sensores,Recepcion Rodete,Recepcion Tableros,Recepcion Alabe,Recepcion motor</t>
+  </si>
+  <si>
+    <t>1213459189207079</t>
+  </si>
+  <si>
+    <t>Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>Bodega:,Montaje Alabe</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213459189153328</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe ot 4264</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe ot 4264,Alabe  ot 4264</t>
-  </si>
-  <si>
-    <t>Baja</t>
-  </si>
-  <si>
-    <t>1213459189153329</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe ot 4264</t>
-  </si>
-  <si>
-    <t>Alabe  ot 4264,Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>1213459189153330</t>
-  </si>
-  <si>
-    <t>Tablero ot 4265 - ot 4266</t>
-  </si>
-  <si>
-    <t>Generación OC Tableros  ot 4265 - ot 4266,Fabricación Tablero  ot 4265 - ot 4266</t>
-  </si>
-  <si>
-    <t>1213459189153331</t>
-  </si>
-  <si>
-    <t>Generación OC Tableros  ot 4265 - ot 4266</t>
-  </si>
-  <si>
-    <t>Fabricación Tablero  ot 4265 - ot 4266,Tablero ot 4265 - ot 4266</t>
-  </si>
-  <si>
-    <t>1213459189153332</t>
-  </si>
-  <si>
-    <t>Fabricación Tablero  ot 4265 - ot 4266</t>
-  </si>
-  <si>
-    <t>Tablero ot 4265 - ot 4266,Recepcion Tableros</t>
-  </si>
-  <si>
-    <t>1213459189153336</t>
-  </si>
-  <si>
-    <t>Motor ot 4264</t>
-  </si>
-  <si>
-    <t>Generación OC motor ot 4264,Fabricación motor ot 4264,Planos motor proveedor ot 4264</t>
-  </si>
-  <si>
-    <t>1213459189207060</t>
-  </si>
-  <si>
-    <t>Generación OC motor ot 4264</t>
-  </si>
-  <si>
-    <t>Fabricación motor ot 4264,Motor ot 4264,Planos motor proveedor ot 4264</t>
-  </si>
-  <si>
-    <t>1213459189207061</t>
-  </si>
-  <si>
-    <t>Fabricación motor ot 4264</t>
-  </si>
-  <si>
-    <t>Motor ot 4264,Recepcion motor</t>
-  </si>
-  <si>
-    <t>1213459189207062</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor ot 4264</t>
-  </si>
-  <si>
-    <t>Motor ot 4264,Ingenieria y diseño:,Planos definitivos</t>
-  </si>
-  <si>
-    <t>1213459189153333</t>
-  </si>
-  <si>
-    <t>rodete ot 4264</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete ot 4264,Fabricación Rodete ot 4264</t>
-  </si>
-  <si>
-    <t>1213459189153334</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete ot 4264</t>
-  </si>
-  <si>
-    <t>Fabricación Rodete ot 4264,rodete ot 4264</t>
-  </si>
-  <si>
-    <t>1213459189153335</t>
-  </si>
-  <si>
-    <t>Fabricación Rodete ot 4264</t>
-  </si>
-  <si>
-    <t>rodete ot 4264,Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>1213459189207063</t>
-  </si>
-  <si>
-    <t>Materiales a codigo // compras locales aprovisionamientomiento:</t>
-  </si>
-  <si>
-    <t>Yerlia Ayleen Castillo Diaz</t>
-  </si>
-  <si>
-    <t>yerlia.castillo@zitron.com</t>
-  </si>
-  <si>
-    <t>Generación OC materiales,Fabricacion a codigo y compras locales</t>
-  </si>
-  <si>
-    <t>1213459189207064</t>
-  </si>
-  <si>
-    <t>Generación OC materiales</t>
-  </si>
-  <si>
-    <t>Fabricacion a codigo y compras locales,Materiales a codigo // compras locales aprovisionamientomiento:</t>
-  </si>
-  <si>
-    <t>1213459189207065</t>
-  </si>
-  <si>
-    <t>Fabricacion a codigo y compras locales</t>
-  </si>
-  <si>
-    <t>Materiales a codigo // compras locales aprovisionamientomiento:,Recepcion materiales a codigos // compras locales aprovisionamiento</t>
-  </si>
-  <si>
-    <t>1213458788103037</t>
-  </si>
-  <si>
-    <t>Sensores</t>
-  </si>
-  <si>
-    <t>Generación OC Sensores,Fabricacion Sensores</t>
-  </si>
-  <si>
-    <t>1213458788103039</t>
-  </si>
-  <si>
-    <t>Generación OC Sensores</t>
-  </si>
-  <si>
-    <t>Fabricacion Sensores,Sensores</t>
-  </si>
-  <si>
-    <t>1213458788103040</t>
-  </si>
-  <si>
-    <t>Fabricacion Sensores</t>
-  </si>
-  <si>
-    <t>Sensores,Recepcion Sensores</t>
-  </si>
-  <si>
-    <t>1213459189207066</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseño:</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor ot 4264,Planos preliminar,Check plano,Check pruebas FAT</t>
-  </si>
-  <si>
-    <t>1213459189207067</t>
-  </si>
-  <si>
-    <t>Planos preliminar</t>
-  </si>
-  <si>
-    <t>Hernan Roberto Gutierrez Barrientos</t>
-  </si>
-  <si>
-    <t>hgutierrez@zitron.com</t>
-  </si>
-  <si>
-    <t>Ingenieria y diseño:,Planos definitivos,Ingenieria Y diseño</t>
-  </si>
-  <si>
-    <t>1213459189207068</t>
-  </si>
-  <si>
-    <t>Planos definitivos</t>
-  </si>
-  <si>
-    <t>Francisca González Cornejo</t>
-  </si>
-  <si>
-    <t>francisca.gonzalez@zitron.com</t>
-  </si>
-  <si>
-    <t>Planos preliminar,Planos motor proveedor ot 4264</t>
-  </si>
-  <si>
-    <t>Check plano</t>
-  </si>
-  <si>
-    <t>1213560053852552</t>
-  </si>
-  <si>
-    <t>Armado,Control de calidad Armado,Ingenieria y diseño:,Montaje motor,Montaje Alabe,Montaje Rodete,Montaje sensor</t>
-  </si>
-  <si>
-    <t>1213560053852553</t>
-  </si>
-  <si>
-    <t>Check pruebas FAT</t>
-  </si>
-  <si>
-    <t>Pruebas FAT</t>
-  </si>
-  <si>
-    <t>RE-PINTADO,Ingenieria y diseño:</t>
-  </si>
-  <si>
-    <t>1213459189207069</t>
-  </si>
-  <si>
-    <t>Bodega:</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Recepcion materiales a codigos // compras locales aprovisionamiento</t>
-  </si>
-  <si>
-    <t>1213459189207070</t>
-  </si>
-  <si>
-    <t>Recepcion materiales a codigos // compras locales aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Victor Muñoz</t>
-  </si>
-  <si>
-    <t>victor.munoz@zitron.com</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Bodega:</t>
-  </si>
-  <si>
-    <t>1213459189207071</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Nicolás López</t>
-  </si>
-  <si>
-    <t>nicolas.lopez@zitron.com</t>
-  </si>
-  <si>
-    <t>Bodega:,Preparación Materiales</t>
-  </si>
-  <si>
-    <t>1213459189207072</t>
-  </si>
-  <si>
-    <t>Caldereria:</t>
-  </si>
-  <si>
-    <t>Preparación Materiales</t>
-  </si>
-  <si>
-    <t>1213459189207073</t>
-  </si>
-  <si>
-    <t>Nicolás Mol</t>
-  </si>
-  <si>
-    <t>nicolas.mol@zitron.com</t>
-  </si>
-  <si>
-    <t>Caldereria:,Armado,Armado</t>
-  </si>
-  <si>
-    <t>1213459189207074</t>
-  </si>
-  <si>
-    <t>Armado</t>
-  </si>
-  <si>
-    <t>Preparación Materiales,Check plano</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>1213459189207075</t>
-  </si>
-  <si>
-    <t>Armado,Check plano</t>
-  </si>
-  <si>
-    <t>Revestimiento</t>
-  </si>
-  <si>
-    <t>1213459189207076</t>
-  </si>
-  <si>
-    <t>Recepcion Sensores,Recepcion Rodete,Recepcion Tableros,Recepcion Alabe,Recepcion motor</t>
-  </si>
-  <si>
-    <t>1213459189207079</t>
-  </si>
-  <si>
-    <t>Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>Bodega:,Montaje Alabe</t>
   </si>
   <si>
     <t>1213459189207078</t>
@@ -3023,7 +3023,7 @@
         <v>46191.874819687495</v>
       </c>
       <c r="D28" s="5">
-        <v>46204.193195381944</v>
+        <v>46212.17176924768</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>109</v>
@@ -3073,13 +3073,13 @@
       <c r="T28" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U28" s="12" t="s">
-        <v>113</v>
+      <c r="U28" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B29" s="8">
         <v>46079.83530212963</v>
@@ -3091,7 +3091,7 @@
         <v>46169.848412384265</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>26</v>
@@ -3124,7 +3124,7 @@
         <v>83</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="Q29" s="9"/>
       <c r="R29" s="9"/>
@@ -3135,12 +3135,12 @@
         <v>58</v>
       </c>
       <c r="U29" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B30" s="5">
         <v>46079.83530236111</v>
@@ -3152,7 +3152,7 @@
         <v>46191.87480704861</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
@@ -3182,10 +3182,10 @@
         <v>109</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
@@ -3196,12 +3196,12 @@
         <v>58</v>
       </c>
       <c r="U30" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B31" s="8">
         <v>46079.83530269676</v>
@@ -3213,7 +3213,7 @@
         <v>46198.19648104167</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>26</v>
@@ -3243,7 +3243,7 @@
         <v>106</v>
       </c>
       <c r="O31" s="9" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P31" s="9" t="s">
         <v>106</v>
@@ -3266,7 +3266,7 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B32" s="5">
         <v>46079.83530295139</v>
@@ -3278,7 +3278,7 @@
         <v>46182.6792266088</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
@@ -3305,13 +3305,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O32" s="6" t="s">
         <v>89</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
@@ -3322,12 +3322,12 @@
         <v>58</v>
       </c>
       <c r="U32" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B33" s="8">
         <v>46079.83530319444</v>
@@ -3339,7 +3339,7 @@
         <v>46191.874698125</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>26</v>
@@ -3366,13 +3366,13 @@
         <v>26</v>
       </c>
       <c r="N33" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P33" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="Q33" s="9"/>
       <c r="R33" s="9"/>
@@ -3383,12 +3383,12 @@
         <v>58</v>
       </c>
       <c r="U33" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B34" s="5">
         <v>46079.835301238425</v>
@@ -3400,7 +3400,7 @@
         <v>46191.874603414355</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
@@ -3430,7 +3430,7 @@
         <v>106</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="P34" s="6" t="s">
         <v>106</v>
@@ -3453,7 +3453,7 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B35" s="8">
         <v>46079.835301493054</v>
@@ -3465,7 +3465,7 @@
         <v>46169.84848269676</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>26</v>
@@ -3492,13 +3492,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="O35" s="9" t="s">
         <v>86</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="Q35" s="9"/>
       <c r="R35" s="9"/>
@@ -3509,12 +3509,12 @@
         <v>58</v>
       </c>
       <c r="U35" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B36" s="5">
         <v>46079.83530179398</v>
@@ -3526,7 +3526,7 @@
         <v>46191.87457655092</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
@@ -3553,13 +3553,13 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
@@ -3570,12 +3570,12 @@
         <v>58</v>
       </c>
       <c r="U36" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B37" s="8">
         <v>46079.83530215277</v>
@@ -3587,7 +3587,7 @@
         <v>46169.84849621527</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>26</v>
@@ -3614,13 +3614,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="O37" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="Q37" s="9"/>
       <c r="R37" s="9"/>
@@ -3631,12 +3631,12 @@
         <v>58</v>
       </c>
       <c r="U37" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B38" s="5">
         <v>46079.83530342593</v>
@@ -3648,7 +3648,7 @@
         <v>46191.875013136574</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
@@ -3678,7 +3678,7 @@
         <v>106</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>106</v>
@@ -3701,7 +3701,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B39" s="8">
         <v>46079.83530366898</v>
@@ -3713,7 +3713,7 @@
         <v>46191.87447540509</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>26</v>
@@ -3740,13 +3740,13 @@
         <v>26</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O39" s="9" t="s">
         <v>92</v>
       </c>
       <c r="P39" s="9" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="Q39" s="9"/>
       <c r="R39" s="9"/>
@@ -3757,12 +3757,12 @@
         <v>58</v>
       </c>
       <c r="U39" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B40" s="5">
         <v>46079.83530085648</v>
@@ -3774,7 +3774,7 @@
         <v>46191.87498288194</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
@@ -3801,13 +3801,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
@@ -3818,12 +3818,12 @@
         <v>58</v>
       </c>
       <c r="U40" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B41" s="8">
         <v>46079.835302418986</v>
@@ -3835,16 +3835,16 @@
         <v>46191.874875995374</v>
       </c>
       <c r="E41" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="F41" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G41" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="F41" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G41" s="9" t="s">
+      <c r="H41" s="9" t="s">
         <v>153</v>
-      </c>
-      <c r="H41" s="9" t="s">
-        <v>154</v>
       </c>
       <c r="I41" s="8">
         <v>46097</v>
@@ -3865,7 +3865,7 @@
         <v>106</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="P41" s="9" t="s">
         <v>106</v>
@@ -3888,7 +3888,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B42" s="5">
         <v>46079.83530269676</v>
@@ -3900,16 +3900,16 @@
         <v>46209.779950625</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="H42" s="6" t="s">
         <v>153</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>154</v>
       </c>
       <c r="I42" s="5">
         <v>46097</v>
@@ -3927,13 +3927,13 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>96</v>
       </c>
       <c r="P42" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="Q42" s="6"/>
       <c r="R42" s="6"/>
@@ -3944,12 +3944,12 @@
         <v>58</v>
       </c>
       <c r="U42" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B43" s="8">
         <v>46079.835302962965</v>
@@ -3961,16 +3961,16 @@
         <v>46114.765690740736</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="H43" s="9" t="s">
         <v>153</v>
-      </c>
-      <c r="H43" s="9" t="s">
-        <v>154</v>
       </c>
       <c r="I43" s="8">
         <v>46115</v>
@@ -3988,13 +3988,13 @@
         <v>26</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="P43" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="Q43" s="9"/>
       <c r="R43" s="9"/>
@@ -4005,12 +4005,12 @@
         <v>58</v>
       </c>
       <c r="U43" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B44" s="5">
         <v>46079.87449113426</v>
@@ -4022,16 +4022,16 @@
         <v>46204.18561212963</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="H44" s="6" t="s">
         <v>153</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>154</v>
       </c>
       <c r="I44" s="5">
         <v>46097</v>
@@ -4052,7 +4052,7 @@
         <v>106</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="P44" s="6" t="s">
         <v>106</v>
@@ -4075,7 +4075,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B45" s="8">
         <v>46079.87456693287</v>
@@ -4087,16 +4087,16 @@
         <v>46191.80111972222</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="H45" s="9" t="s">
         <v>153</v>
-      </c>
-      <c r="H45" s="9" t="s">
-        <v>154</v>
       </c>
       <c r="I45" s="8">
         <v>46097</v>
@@ -4114,13 +4114,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="O45" s="9" t="s">
         <v>101</v>
       </c>
       <c r="P45" s="9" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="Q45" s="9"/>
       <c r="R45" s="9"/>
@@ -4131,12 +4131,12 @@
         <v>58</v>
       </c>
       <c r="U45" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B46" s="5">
         <v>46079.8746696875</v>
@@ -4148,16 +4148,16 @@
         <v>46114.766096481486</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G46" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="H46" s="6" t="s">
         <v>153</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>154</v>
       </c>
       <c r="I46" s="5">
         <v>46126</v>
@@ -4175,13 +4175,13 @@
         <v>26</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="P46" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Q46" s="6"/>
       <c r="R46" s="6"/>
@@ -4192,12 +4192,12 @@
         <v>58</v>
       </c>
       <c r="U46" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B47" s="8">
         <v>46079.835303252315</v>
@@ -4207,7 +4207,7 @@
         <v>46127.68782663194</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>25</v>
@@ -4231,7 +4231,7 @@
         <v>26</v>
       </c>
       <c r="O47" s="9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="P47" s="9" t="s">
         <v>26</v>
@@ -4246,7 +4246,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B48" s="5">
         <v>46079.8353035301</v>
@@ -4258,16 +4258,16 @@
         <v>46114.79548327546</v>
       </c>
       <c r="E48" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G48" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="F48" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G48" s="6" t="s">
+      <c r="H48" s="6" t="s">
         <v>176</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>177</v>
       </c>
       <c r="I48" s="5">
         <v>46093</v>
@@ -4285,13 +4285,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>69</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="Q48" s="5">
         <v>46093</v>
@@ -4311,7 +4311,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B49" s="8">
         <v>46079.83530068287</v>
@@ -4323,16 +4323,16 @@
         <v>46156.20046739583</v>
       </c>
       <c r="E49" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="F49" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G49" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="F49" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G49" s="9" t="s">
+      <c r="H49" s="9" t="s">
         <v>181</v>
-      </c>
-      <c r="H49" s="9" t="s">
-        <v>182</v>
       </c>
       <c r="I49" s="8">
         <v>46149</v>
@@ -4350,13 +4350,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="O49" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="P49" s="9" t="s">
         <v>183</v>
-      </c>
-      <c r="P49" s="9" t="s">
-        <v>184</v>
       </c>
       <c r="Q49" s="8">
         <v>46149</v>
@@ -4376,7 +4376,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B50" s="5">
         <v>46087.628862847225</v>
@@ -4388,16 +4388,16 @@
         <v>46158.99592378472</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G50" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="H50" s="6" t="s">
         <v>176</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>177</v>
       </c>
       <c r="I50" s="5">
         <v>46156</v>
@@ -4415,13 +4415,13 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="P50" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="Q50" s="5">
         <v>46156</v>
@@ -4441,7 +4441,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B51" s="8">
         <v>46087.62890292824</v>
@@ -4451,16 +4451,16 @@
         <v>46127.69021349537</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G51" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="H51" s="9" t="s">
         <v>181</v>
-      </c>
-      <c r="H51" s="9" t="s">
-        <v>182</v>
       </c>
       <c r="I51" s="8">
         <v>46243</v>
@@ -4478,13 +4478,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="O51" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="P51" s="9" t="s">
         <v>189</v>
-      </c>
-      <c r="P51" s="9" t="s">
-        <v>190</v>
       </c>
       <c r="Q51" s="8">
         <v>46243</v>
@@ -4499,22 +4499,24 @@
         <v>58</v>
       </c>
       <c r="U51" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B52" s="5">
         <v>46079.835301053245</v>
       </c>
-      <c r="C52" s="6"/>
+      <c r="C52" s="5">
+        <v>46211.896528136574</v>
+      </c>
       <c r="D52" s="5">
-        <v>46209.78807094907</v>
+        <v>46211.90007753472</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>25</v>
@@ -4538,26 +4540,24 @@
         <v>26</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="P52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
-      <c r="S52" s="6">
-        <v>1</v>
-      </c>
+      <c r="S52" s="6"/>
       <c r="T52" s="10" t="s">
         <v>31</v>
       </c>
       <c r="U52" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B53" s="8">
         <v>46079.835301342595</v>
@@ -4569,16 +4569,16 @@
         <v>46209.78806449074</v>
       </c>
       <c r="E53" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G53" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="F53" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G53" s="9" t="s">
+      <c r="H53" s="9" t="s">
         <v>196</v>
-      </c>
-      <c r="H53" s="9" t="s">
-        <v>197</v>
       </c>
       <c r="I53" s="8">
         <v>46147</v>
@@ -4596,13 +4596,13 @@
         <v>26</v>
       </c>
       <c r="N53" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O53" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="P53" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="Q53" s="8">
         <v>46147</v>
@@ -4622,26 +4622,26 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B54" s="5">
         <v>46079.83530162037</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46209.78806983796</v>
+        <v>46211.896555671294</v>
       </c>
       <c r="E54" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G54" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="F54" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G54" s="6" t="s">
+      <c r="H54" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="H54" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="I54" s="5">
         <v>46149</v>
@@ -4659,13 +4659,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Q54" s="5">
         <v>46149</v>
@@ -4676,8 +4676,8 @@
       <c r="S54" s="6">
         <v>1</v>
       </c>
-      <c r="T54" s="12" t="s">
-        <v>81</v>
+      <c r="T54" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U54" s="11" t="s">
         <v>32</v>
@@ -4685,7 +4685,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B55" s="8">
         <v>46079.835301886575</v>
@@ -4695,7 +4695,7 @@
         <v>46080.57920532407</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>25</v>
@@ -4719,7 +4719,7 @@
         <v>26</v>
       </c>
       <c r="O55" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="P55" s="9" t="s">
         <v>26</v>
@@ -4733,31 +4733,31 @@
         <v>58</v>
       </c>
       <c r="U55" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B56" s="5">
         <v>46079.835302164356</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46209.79160884259</v>
+        <v>46211.89656313657</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="H56" s="6" t="s">
         <v>208</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>209</v>
       </c>
       <c r="I56" s="5">
         <v>46153</v>
@@ -4775,13 +4775,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="Q56" s="5">
         <v>46153</v>
@@ -4801,7 +4801,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B57" s="8">
         <v>46079.835302418986</v>
@@ -4811,16 +4811,16 @@
         <v>46191.1671537963</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="H57" s="9" t="s">
         <v>208</v>
-      </c>
-      <c r="H57" s="9" t="s">
-        <v>209</v>
       </c>
       <c r="I57" s="8">
         <v>46162</v>
@@ -4838,13 +4838,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O57" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="P57" s="9" t="s">
         <v>213</v>
-      </c>
-      <c r="P57" s="9" t="s">
-        <v>214</v>
       </c>
       <c r="Q57" s="8">
         <v>46162</v>
@@ -4864,7 +4864,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B58" s="5">
         <v>46079.835302673615</v>
@@ -4874,16 +4874,16 @@
         <v>46193.205434930554</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="H58" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="H58" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="I58" s="5">
         <v>46191</v>
@@ -4901,13 +4901,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O58" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="P58" s="6" t="s">
         <v>216</v>
-      </c>
-      <c r="P58" s="6" t="s">
-        <v>217</v>
       </c>
       <c r="Q58" s="5">
         <v>46191</v>
@@ -4927,7 +4927,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B59" s="8">
         <v>46079.83530291667</v>
@@ -4937,7 +4937,7 @@
         <v>46158.99585525463</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>25</v>
@@ -4961,7 +4961,7 @@
         <v>26</v>
       </c>
       <c r="O59" s="9" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="P59" s="9" t="s">
         <v>26</v>
@@ -4975,12 +4975,12 @@
         <v>58</v>
       </c>
       <c r="U59" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B60" s="5">
         <v>46079.83530225694</v>
@@ -4990,16 +4990,16 @@
         <v>46210.81198283564</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="H60" s="6" t="s">
         <v>196</v>
-      </c>
-      <c r="H60" s="6" t="s">
-        <v>197</v>
       </c>
       <c r="I60" s="5">
         <v>46212</v>
@@ -5017,13 +5017,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="Q60" s="5">
         <v>46212</v>
@@ -5038,7 +5038,7 @@
         <v>81</v>
       </c>
       <c r="U60" s="12" t="s">
-        <v>113</v>
+        <v>222</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -5059,10 +5059,10 @@
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="H61" s="9" t="s">
         <v>196</v>
-      </c>
-      <c r="H61" s="9" t="s">
-        <v>197</v>
       </c>
       <c r="I61" s="8">
         <v>46198</v>
@@ -5080,10 +5080,10 @@
         <v>26</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O61" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="P61" s="9" t="s">
         <v>224</v>
@@ -5122,10 +5122,10 @@
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="H62" s="6" t="s">
         <v>196</v>
-      </c>
-      <c r="H62" s="6" t="s">
-        <v>197</v>
       </c>
       <c r="I62" s="5">
         <v>46204</v>
@@ -5143,10 +5143,10 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>227</v>
@@ -5185,10 +5185,10 @@
         <v>26</v>
       </c>
       <c r="G63" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="H63" s="9" t="s">
         <v>196</v>
-      </c>
-      <c r="H63" s="9" t="s">
-        <v>197</v>
       </c>
       <c r="I63" s="8">
         <v>46149</v>
@@ -5206,10 +5206,10 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O63" s="9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="P63" s="9" t="s">
         <v>230</v>
@@ -5248,10 +5248,10 @@
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="H64" s="6" t="s">
         <v>196</v>
-      </c>
-      <c r="H64" s="6" t="s">
-        <v>197</v>
       </c>
       <c r="I64" s="5">
         <v>46234</v>
@@ -5269,10 +5269,10 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="P64" s="6" t="s">
         <v>233</v>
@@ -5290,7 +5290,7 @@
         <v>81</v>
       </c>
       <c r="U64" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -5343,7 +5343,7 @@
         <v>58</v>
       </c>
       <c r="U65" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
@@ -5355,10 +5355,10 @@
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46205.19330442129</v>
+        <v>46212.167524178236</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
@@ -5388,7 +5388,7 @@
         <v>235</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>238</v>
@@ -5406,7 +5406,7 @@
         <v>58</v>
       </c>
       <c r="U66" s="12" t="s">
-        <v>113</v>
+        <v>222</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -5469,7 +5469,7 @@
         <v>58</v>
       </c>
       <c r="U67" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5532,7 +5532,7 @@
         <v>58</v>
       </c>
       <c r="U68" s="12" t="s">
-        <v>113</v>
+        <v>222</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46127.68782931713</v>
+        <v>46212.201619583335</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>248</v>
@@ -5594,8 +5594,8 @@
       <c r="T69" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="U69" s="10" t="s">
-        <v>117</v>
+      <c r="U69" s="12" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
@@ -5658,7 +5658,7 @@
         <v>58</v>
       </c>
       <c r="U70" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
@@ -5673,7 +5673,7 @@
         <v>46158.99592372685</v>
       </c>
       <c r="E71" s="9" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F71" s="9" t="s">
         <v>26</v>
@@ -5721,7 +5721,7 @@
         <v>58</v>
       </c>
       <c r="U71" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -5766,7 +5766,7 @@
         <v>235</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>258</v>
@@ -5784,7 +5784,7 @@
         <v>58</v>
       </c>
       <c r="U72" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -5892,7 +5892,7 @@
         <v>58</v>
       </c>
       <c r="U74" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -5955,7 +5955,7 @@
         <v>58</v>
       </c>
       <c r="U75" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -5976,10 +5976,10 @@
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="H76" s="6" t="s">
         <v>208</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>209</v>
       </c>
       <c r="I76" s="5">
         <v>46251</v>
@@ -6018,7 +6018,7 @@
         <v>58</v>
       </c>
       <c r="U76" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -6039,10 +6039,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="H77" s="9" t="s">
         <v>208</v>
-      </c>
-      <c r="H77" s="9" t="s">
-        <v>209</v>
       </c>
       <c r="I77" s="8">
         <v>46252</v>
@@ -6081,7 +6081,7 @@
         <v>58</v>
       </c>
       <c r="U77" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
@@ -6191,7 +6191,7 @@
         <v>58</v>
       </c>
       <c r="U79" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -6254,7 +6254,7 @@
         <v>58</v>
       </c>
       <c r="U80" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
@@ -6307,7 +6307,7 @@
         <v>58</v>
       </c>
       <c r="U81" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
@@ -6370,7 +6370,7 @@
         <v>58</v>
       </c>
       <c r="U82" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
@@ -6433,7 +6433,7 @@
         <v>58</v>
       </c>
       <c r="U83" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-07-13 13:08 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -5607,7 +5607,7 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46127.687829814815</v>
+        <v>46216.19986287037</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>251</v>
@@ -5657,8 +5657,8 @@
       <c r="T70" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="U70" s="10" t="s">
-        <v>116</v>
+      <c r="U70" s="12" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-07-13 19:47 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -4934,7 +4934,7 @@
       </c>
       <c r="C59" s="9"/>
       <c r="D59" s="8">
-        <v>46158.99585525463</v>
+        <v>46216.76549305556</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>191</v>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="8">
-        <v>46200.20831664352</v>
+        <v>46216.766091377314</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>56</v>
@@ -5111,9 +5111,11 @@
       <c r="B62" s="5">
         <v>46079.87589787037</v>
       </c>
-      <c r="C62" s="6"/>
+      <c r="C62" s="5">
+        <v>46216.76548623842</v>
+      </c>
       <c r="D62" s="5">
-        <v>46206.16743369213</v>
+        <v>46216.765501898146</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>225</v>
@@ -5158,10 +5160,10 @@
         <v>46205</v>
       </c>
       <c r="S62" s="6">
-        <v>0</v>
-      </c>
-      <c r="T62" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="T62" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U62" s="11" t="s">
         <v>32</v>
@@ -5237,9 +5239,11 @@
       <c r="B64" s="5">
         <v>46079.83530262731</v>
       </c>
-      <c r="C64" s="6"/>
+      <c r="C64" s="5">
+        <v>46216.7654346412</v>
+      </c>
       <c r="D64" s="5">
-        <v>46191.874584930556</v>
+        <v>46216.765453831016</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>231</v>
@@ -5284,10 +5288,10 @@
         <v>46237</v>
       </c>
       <c r="S64" s="6">
-        <v>0</v>
-      </c>
-      <c r="T64" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="T64" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U64" s="10" t="s">
         <v>116</v>
@@ -5418,7 +5422,7 @@
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="8">
-        <v>46127.6878281713</v>
+        <v>46216.76544502315</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>239</v>
@@ -5607,7 +5611,7 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46216.19986287037</v>
+        <v>46216.765493900464</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>251</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-14 21:13 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -4513,7 +4513,7 @@
         <v>46211.896528136574</v>
       </c>
       <c r="D52" s="5">
-        <v>46211.90007753472</v>
+        <v>46217.8196680324</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>191</v>
@@ -4548,8 +4548,8 @@
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
       <c r="S52" s="6"/>
-      <c r="T52" s="10" t="s">
-        <v>31</v>
+      <c r="T52" s="12" t="s">
+        <v>81</v>
       </c>
       <c r="U52" s="10" t="s">
         <v>116</v>
@@ -4627,9 +4627,11 @@
       <c r="B54" s="5">
         <v>46079.83530162037</v>
       </c>
-      <c r="C54" s="6"/>
+      <c r="C54" s="5">
+        <v>46217.81965075231</v>
+      </c>
       <c r="D54" s="5">
-        <v>46211.896555671294</v>
+        <v>46217.81965280093</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>199</v>
@@ -4745,7 +4747,7 @@
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46211.89656313657</v>
+        <v>46217.81965958333</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>205</v>
@@ -5050,7 +5052,7 @@
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="8">
-        <v>46216.766091377314</v>
+        <v>46217.768278020834</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>56</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-17 14:52 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -761,16 +761,16 @@
     <t>Montaje Alabe,Revestimiento,Recepcion Rodete,Check plano</t>
   </si>
   <si>
+    <t>1213458788103121</t>
+  </si>
+  <si>
+    <t>Montaje sensor</t>
+  </si>
+  <si>
+    <t>Revestimiento,Recepcion Sensores,Check plano</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213458788103121</t>
-  </si>
-  <si>
-    <t>Montaje sensor</t>
-  </si>
-  <si>
-    <t>Revestimiento,Recepcion Sensores,Check plano</t>
   </si>
   <si>
     <t>1213459189207086</t>
@@ -5531,7 +5531,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46212.201619583335</v>
+        <v>46220.2056790625</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>244</v>
@@ -5579,13 +5579,13 @@
       <c r="T69" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="U69" s="12" t="s">
-        <v>246</v>
+      <c r="U69" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B70" s="5">
         <v>46080.49271868056</v>
@@ -5595,7 +5595,7 @@
         <v>46216.765493900464</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
@@ -5623,7 +5623,7 @@
         <v>231</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>238</v>
@@ -5641,7 +5641,7 @@
         <v>58</v>
       </c>
       <c r="U70" s="12" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-07-21 12:45 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1038" uniqueCount="291">
   <si>
     <t>50001518 - EQ. CHAPARRAL</t>
   </si>
@@ -771,9 +771,6 @@
   </si>
   <si>
     <t>Revestimiento,Recepcion Sensores,Check plano</t>
-  </si>
-  <si>
-    <t>Media</t>
   </si>
   <si>
     <t>1213459189207086</t>
@@ -5607,7 +5604,7 @@
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46223.80773064814</v>
+        <v>46224.20075512731</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>248</v>
@@ -5657,13 +5654,13 @@
       <c r="T70" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="U70" s="12" t="s">
-        <v>250</v>
+      <c r="U70" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B71" s="8">
         <v>46079.83530460648</v>
@@ -5703,10 +5700,10 @@
         <v>232</v>
       </c>
       <c r="O71" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="P71" s="9" t="s">
         <v>252</v>
-      </c>
-      <c r="P71" s="9" t="s">
-        <v>253</v>
       </c>
       <c r="Q71" s="8">
         <v>46240</v>
@@ -5726,7 +5723,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B72" s="5">
         <v>46079.83530493056</v>
@@ -5736,7 +5733,7 @@
         <v>46223.807729548615</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
@@ -5769,7 +5766,7 @@
         <v>185</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="Q72" s="5">
         <v>46244</v>
@@ -5789,7 +5786,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B73" s="8">
         <v>46079.83530144676</v>
@@ -5799,7 +5796,7 @@
         <v>46090.67671023148</v>
       </c>
       <c r="E73" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F73" s="9" t="s">
         <v>25</v>
@@ -5823,7 +5820,7 @@
         <v>26</v>
       </c>
       <c r="O73" s="9" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="P73" s="9" t="s">
         <v>26</v>
@@ -5836,7 +5833,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B74" s="5">
         <v>46079.83530181713</v>
@@ -5846,16 +5843,16 @@
         <v>46210.61678060185</v>
       </c>
       <c r="E74" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G74" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="F74" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G74" s="6" t="s">
+      <c r="H74" s="6" t="s">
         <v>262</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>263</v>
       </c>
       <c r="I74" s="6"/>
       <c r="J74" s="5">
@@ -5871,13 +5868,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="Q74" s="5">
         <v>46245</v>
@@ -5897,7 +5894,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B75" s="8">
         <v>46079.8353024074</v>
@@ -5934,13 +5931,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O75" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="P75" s="9" t="s">
         <v>266</v>
-      </c>
-      <c r="P75" s="9" t="s">
-        <v>267</v>
       </c>
       <c r="Q75" s="8">
         <v>46246</v>
@@ -5960,7 +5957,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B76" s="5">
         <v>46079.83530269676</v>
@@ -5970,7 +5967,7 @@
         <v>46090.80487153935</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>26</v>
@@ -5997,13 +5994,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O76" s="6" t="s">
         <v>57</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="Q76" s="5">
         <v>46251</v>
@@ -6023,7 +6020,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B77" s="8">
         <v>46079.83530306713</v>
@@ -6033,7 +6030,7 @@
         <v>46090.80495936342</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>26</v>
@@ -6060,13 +6057,13 @@
         <v>26</v>
       </c>
       <c r="N77" s="9" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="P77" s="9" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="Q77" s="8">
         <v>46252</v>
@@ -6086,7 +6083,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B78" s="5">
         <v>46079.83530333333</v>
@@ -6096,7 +6093,7 @@
         <v>46090.67667782407</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>25</v>
@@ -6120,7 +6117,7 @@
         <v>26</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>26</v>
@@ -6133,7 +6130,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B79" s="8">
         <v>46079.83530363426</v>
@@ -6143,16 +6140,16 @@
         <v>46090.805033425924</v>
       </c>
       <c r="E79" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="F79" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G79" s="9" t="s">
         <v>278</v>
       </c>
-      <c r="F79" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G79" s="9" t="s">
+      <c r="H79" s="9" t="s">
         <v>279</v>
-      </c>
-      <c r="H79" s="9" t="s">
-        <v>280</v>
       </c>
       <c r="I79" s="8">
         <v>46253</v>
@@ -6170,13 +6167,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="Q79" s="8">
         <v>46252</v>
@@ -6196,7 +6193,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B80" s="5">
         <v>46079.83530395833</v>
@@ -6206,16 +6203,16 @@
         <v>46114.51489402778</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="H80" s="6" t="s">
         <v>279</v>
-      </c>
-      <c r="H80" s="6" t="s">
-        <v>280</v>
       </c>
       <c r="I80" s="5">
         <v>46253</v>
@@ -6233,13 +6230,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="Q80" s="5">
         <v>46252</v>
@@ -6259,7 +6256,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B81" s="8">
         <v>46090.6740474074</v>
@@ -6269,7 +6266,7 @@
         <v>46090.6782175</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>25</v>
@@ -6293,7 +6290,7 @@
         <v>26</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="P81" s="9" t="s">
         <v>26</v>
@@ -6312,7 +6309,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B82" s="5">
         <v>46090.674231365745</v>
@@ -6322,7 +6319,7 @@
         <v>46090.80510871528</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
@@ -6349,13 +6346,13 @@
         <v>26</v>
       </c>
       <c r="N82" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="P82" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="Q82" s="5">
         <v>46253</v>
@@ -6375,7 +6372,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="7" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B83" s="8">
         <v>46090.67444209491</v>
@@ -6385,7 +6382,7 @@
         <v>46090.80510556713</v>
       </c>
       <c r="E83" s="9" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F83" s="9" t="s">
         <v>26</v>
@@ -6412,13 +6409,13 @@
         <v>26</v>
       </c>
       <c r="N83" s="9" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="O83" s="9" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="P83" s="9" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="Q83" s="8">
         <v>46262</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-29 15:16 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -5421,7 +5421,7 @@
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="8">
-        <v>46223.80773233796</v>
+        <v>46232.17142269676</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>239</v>
@@ -5471,8 +5471,8 @@
       <c r="T67" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="U67" s="10" t="s">
-        <v>115</v>
+      <c r="U67" s="12" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-02 10:47 Chile
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -596,6 +596,9 @@
     <t>RE-PINTADO,Ingenieria y diseño:</t>
   </si>
   <si>
+    <t>Media</t>
+  </si>
+  <si>
     <t>1213459189207069</t>
   </si>
   <si>
@@ -723,9 +726,6 @@
   </si>
   <si>
     <t>Bodega:,Montaje motor</t>
-  </si>
-  <si>
-    <t>Media</t>
   </si>
   <si>
     <t>1213459189207081</t>
@@ -4451,7 +4451,7 @@
       </c>
       <c r="C51" s="9"/>
       <c r="D51" s="8">
-        <v>46127.69021349537</v>
+        <v>46236.20194324074</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>188</v>
@@ -4501,13 +4501,13 @@
       <c r="T51" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U51" s="10" t="s">
-        <v>117</v>
+      <c r="U51" s="12" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B52" s="5">
         <v>46079.835301053245</v>
@@ -4519,7 +4519,7 @@
         <v>46217.8196680324</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>25</v>
@@ -4543,7 +4543,7 @@
         <v>26</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="P52" s="6" t="s">
         <v>26</v>
@@ -4560,7 +4560,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B53" s="8">
         <v>46079.835301342595</v>
@@ -4572,16 +4572,16 @@
         <v>46209.78806449074</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H53" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I53" s="8">
         <v>46147</v>
@@ -4599,13 +4599,13 @@
         <v>26</v>
       </c>
       <c r="N53" s="9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O53" s="9" t="s">
         <v>160</v>
       </c>
       <c r="P53" s="9" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="Q53" s="8">
         <v>46147</v>
@@ -4625,7 +4625,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B54" s="5">
         <v>46079.83530162037</v>
@@ -4637,16 +4637,16 @@
         <v>46217.81965280093</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I54" s="5">
         <v>46149</v>
@@ -4664,13 +4664,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q54" s="5">
         <v>46149</v>
@@ -4690,7 +4690,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B55" s="8">
         <v>46079.835301886575</v>
@@ -4700,7 +4700,7 @@
         <v>46080.57920532407</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>25</v>
@@ -4724,7 +4724,7 @@
         <v>26</v>
       </c>
       <c r="O55" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="P55" s="9" t="s">
         <v>26</v>
@@ -4743,7 +4743,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B56" s="5">
         <v>46079.835302164356</v>
@@ -4753,16 +4753,16 @@
         <v>46217.81965958333</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I56" s="5">
         <v>46153</v>
@@ -4780,13 +4780,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="Q56" s="5">
         <v>46153</v>
@@ -4806,7 +4806,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="7" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B57" s="8">
         <v>46079.835302418986</v>
@@ -4816,16 +4816,16 @@
         <v>46191.1671537963</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H57" s="9" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I57" s="8">
         <v>46162</v>
@@ -4843,13 +4843,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="O57" s="9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="P57" s="9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Q57" s="8">
         <v>46162</v>
@@ -4869,7 +4869,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B58" s="5">
         <v>46079.835302673615</v>
@@ -4879,16 +4879,16 @@
         <v>46193.205434930554</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I58" s="5">
         <v>46191</v>
@@ -4906,13 +4906,13 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="Q58" s="5">
         <v>46191</v>
@@ -4932,7 +4932,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="7" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B59" s="8">
         <v>46079.83530291667</v>
@@ -4942,7 +4942,7 @@
         <v>46216.76549305556</v>
       </c>
       <c r="E59" s="9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F59" s="9" t="s">
         <v>25</v>
@@ -4966,7 +4966,7 @@
         <v>26</v>
       </c>
       <c r="O59" s="9" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="P59" s="9" t="s">
         <v>26</v>
@@ -4985,7 +4985,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B60" s="5">
         <v>46079.83530225694</v>
@@ -4995,16 +4995,16 @@
         <v>46214.176594108794</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I60" s="5">
         <v>46212</v>
@@ -5022,13 +5022,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>119</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="Q60" s="5">
         <v>46212</v>
@@ -5048,7 +5048,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="7" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B61" s="8">
         <v>46079.835301851854</v>
@@ -5064,10 +5064,10 @@
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I61" s="8">
         <v>46198</v>
@@ -5085,13 +5085,13 @@
         <v>26</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O61" s="9" t="s">
         <v>128</v>
       </c>
       <c r="P61" s="9" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="Q61" s="8">
         <v>46198</v>
@@ -5111,7 +5111,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B62" s="5">
         <v>46079.87589787037</v>
@@ -5123,16 +5123,16 @@
         <v>46216.765501898146</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F62" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I62" s="5">
         <v>46204</v>
@@ -5150,13 +5150,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>169</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="Q62" s="5">
         <v>46204</v>
@@ -5176,7 +5176,7 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="7" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B63" s="8">
         <v>46079.83530319444</v>
@@ -5186,16 +5186,16 @@
         <v>46191.87499096065</v>
       </c>
       <c r="E63" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G63" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H63" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I63" s="8">
         <v>46149</v>
@@ -5213,13 +5213,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="9" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O63" s="9" t="s">
         <v>149</v>
       </c>
       <c r="P63" s="9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="Q63" s="8">
         <v>46149</v>
@@ -5239,7 +5239,7 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B64" s="5">
         <v>46079.83530262731</v>
@@ -5251,16 +5251,16 @@
         <v>46230.175846087965</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I64" s="5">
         <v>46234</v>
@@ -5278,13 +5278,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O64" s="6" t="s">
         <v>137</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="Q64" s="5">
         <v>46234</v>
@@ -5299,7 +5299,7 @@
         <v>31</v>
       </c>
       <c r="U64" s="12" t="s">
-        <v>234</v>
+        <v>191</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -5367,7 +5367,7 @@
         <v>46223.807732870366</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
@@ -5397,7 +5397,7 @@
         <v>236</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="P66" s="6" t="s">
         <v>239</v>
@@ -5478,7 +5478,7 @@
         <v>116</v>
       </c>
       <c r="U67" s="12" t="s">
-        <v>234</v>
+        <v>191</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5730,7 +5730,7 @@
         <v>116</v>
       </c>
       <c r="U71" s="12" t="s">
-        <v>234</v>
+        <v>191</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -5985,10 +5985,10 @@
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I76" s="5">
         <v>46251</v>
@@ -6048,10 +6048,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H77" s="9" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I77" s="8">
         <v>46252</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-08-12 14:18 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -824,16 +824,16 @@
     <t>Embalaje,Logistica:</t>
   </si>
   <si>
+    <t>1213459189207090</t>
+  </si>
+  <si>
+    <t>Coordinacion Entrega con Cliente,Revisión tableros pruebas</t>
+  </si>
+  <si>
+    <t>PACKING LIST,Logistica:</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213459189207090</t>
-  </si>
-  <si>
-    <t>Coordinacion Entrega con Cliente,Revisión tableros pruebas</t>
-  </si>
-  <si>
-    <t>PACKING LIST,Logistica:</t>
   </si>
   <si>
     <t>1213459189207091</t>
@@ -5828,7 +5828,7 @@
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46245.16728820602</v>
+        <v>46246.17437313657</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>263</v>
@@ -5876,13 +5876,13 @@
       <c r="T74" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U74" s="12" t="s">
-        <v>267</v>
+      <c r="U74" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B75" s="8">
         <v>46079.8353024074</v>
@@ -5922,10 +5922,10 @@
         <v>260</v>
       </c>
       <c r="O75" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="P75" s="9" t="s">
         <v>269</v>
-      </c>
-      <c r="P75" s="9" t="s">
-        <v>270</v>
       </c>
       <c r="Q75" s="8">
         <v>46246</v>
@@ -5940,7 +5940,7 @@
         <v>116</v>
       </c>
       <c r="U75" s="12" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -6003,7 +6003,7 @@
         <v>116</v>
       </c>
       <c r="U76" s="12" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -6066,7 +6066,7 @@
         <v>116</v>
       </c>
       <c r="U77" s="12" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-08-12 21:01 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -4679,7 +4679,7 @@
       </c>
       <c r="C55" s="9"/>
       <c r="D55" s="8">
-        <v>46246.791487766204</v>
+        <v>46246.86788697916</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>205</v>
@@ -4716,8 +4716,8 @@
       <c r="S55" s="9">
         <v>0</v>
       </c>
-      <c r="T55" s="11" t="s">
-        <v>116</v>
+      <c r="T55" s="12" t="s">
+        <v>60</v>
       </c>
       <c r="U55" s="10" t="s">
         <v>117</v>
@@ -4730,9 +4730,11 @@
       <c r="B56" s="5">
         <v>46079.835302164356</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46246.867865057866</v>
+      </c>
       <c r="D56" s="5">
-        <v>46246.791789560186</v>
+        <v>46246.86788344907</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>206</v>
@@ -4777,10 +4779,10 @@
         <v>46161</v>
       </c>
       <c r="S56" s="6">
-        <v>0</v>
-      </c>
-      <c r="T56" s="12" t="s">
-        <v>60</v>
+        <v>1</v>
+      </c>
+      <c r="T56" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U56" s="11" t="s">
         <v>32</v>
@@ -4793,9 +4795,11 @@
       <c r="B57" s="8">
         <v>46079.835302418986</v>
       </c>
-      <c r="C57" s="9"/>
+      <c r="C57" s="8">
+        <v>46246.86958221065</v>
+      </c>
       <c r="D57" s="8">
-        <v>46246.79178846064</v>
+        <v>46246.86959988426</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>212</v>
@@ -4840,10 +4844,10 @@
         <v>46190</v>
       </c>
       <c r="S57" s="9">
-        <v>0</v>
-      </c>
-      <c r="T57" s="12" t="s">
-        <v>60</v>
+        <v>1</v>
+      </c>
+      <c r="T57" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U57" s="11" t="s">
         <v>32</v>
@@ -4858,7 +4862,7 @@
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46237.511034675925</v>
+        <v>46246.86958899305</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>214</v>
@@ -4972,9 +4976,11 @@
       <c r="B60" s="5">
         <v>46079.83530225694</v>
       </c>
-      <c r="C60" s="6"/>
+      <c r="C60" s="5">
+        <v>46246.87366135417</v>
+      </c>
       <c r="D60" s="5">
-        <v>46246.7938296412</v>
+        <v>46246.87366309028</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>221</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-12 17:17 Chile
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="289">
   <si>
     <t>50001518 - EQ. CHAPARRAL</t>
   </si>
@@ -156,6 +156,9 @@
   </si>
   <si>
     <t>Recepcion Tableros,Ingenieria electrica</t>
+  </si>
+  <si>
+    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1213459189153312</t>
@@ -201,9 +204,6 @@
   </si>
   <si>
     <t>Embalaje</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1213459189153314</t>
@@ -1892,7 +1892,7 @@
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46142.66126674769</v>
+        <v>46246.87440424769</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>46</v>
@@ -1927,12 +1927,14 @@
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
       <c r="S10" s="6"/>
-      <c r="T10" s="6"/>
+      <c r="T10" s="12" t="s">
+        <v>48</v>
+      </c>
       <c r="U10" s="6"/>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11" s="8">
         <v>46079.835302858795</v>
@@ -1944,16 +1946,16 @@
         <v>46142.661260625</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I11" s="8">
         <v>46084</v>
@@ -1965,7 +1967,7 @@
         <v>26</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="M11" s="9" t="s">
         <v>26</v>
@@ -1977,7 +1979,7 @@
         <v>40</v>
       </c>
       <c r="P11" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="Q11" s="8">
         <v>46084</v>
@@ -1997,26 +1999,26 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B12" s="5">
         <v>46079.83530313657</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46238.491149560185</v>
+        <v>46246.87971918982</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I12" s="5">
         <v>46202</v>
@@ -2037,10 +2039,10 @@
         <v>46</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q12" s="5">
         <v>46202</v>
@@ -2052,7 +2054,7 @@
         <v>0.1</v>
       </c>
       <c r="T12" s="12" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="U12" s="11" t="s">
         <v>32</v>
@@ -2663,7 +2665,7 @@
         <v>81</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="P22" s="6" t="s">
         <v>91</v>
@@ -3430,7 +3432,7 @@
         <v>1</v>
       </c>
       <c r="T34" s="12" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="U34" s="11" t="s">
         <v>32</v>
@@ -4534,7 +4536,7 @@
       <c r="R52" s="6"/>
       <c r="S52" s="6"/>
       <c r="T52" s="12" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="U52" s="10" t="s">
         <v>117</v>
@@ -4717,7 +4719,7 @@
         <v>0</v>
       </c>
       <c r="T55" s="12" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="U55" s="10" t="s">
         <v>117</v>
@@ -4910,7 +4912,7 @@
         <v>0</v>
       </c>
       <c r="T58" s="12" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="U58" s="11" t="s">
         <v>32</v>
@@ -4925,7 +4927,7 @@
       </c>
       <c r="C59" s="9"/>
       <c r="D59" s="8">
-        <v>46244.07001476852</v>
+        <v>46246.87439424769</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>192</v>
@@ -4976,11 +4978,9 @@
       <c r="B60" s="5">
         <v>46079.83530225694</v>
       </c>
-      <c r="C60" s="5">
-        <v>46246.87366135417</v>
-      </c>
+      <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46246.87366309028</v>
+        <v>46246.87417596065</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>221</v>
@@ -5025,10 +5025,10 @@
         <v>46213</v>
       </c>
       <c r="S60" s="6">
-        <v>0</v>
-      </c>
-      <c r="T60" s="12" t="s">
-        <v>60</v>
+        <v>1</v>
+      </c>
+      <c r="T60" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U60" s="11" t="s">
         <v>32</v>
@@ -5041,12 +5041,14 @@
       <c r="B61" s="8">
         <v>46079.835301851854</v>
       </c>
-      <c r="C61" s="9"/>
+      <c r="C61" s="8">
+        <v>46246.874389398145</v>
+      </c>
       <c r="D61" s="8">
-        <v>46217.768278020834</v>
+        <v>46246.87440410879</v>
       </c>
       <c r="E61" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F61" s="9" t="s">
         <v>26</v>
@@ -5088,10 +5090,10 @@
         <v>46199</v>
       </c>
       <c r="S61" s="9">
-        <v>0</v>
-      </c>
-      <c r="T61" s="12" t="s">
-        <v>60</v>
+        <v>1</v>
+      </c>
+      <c r="T61" s="10" t="s">
+        <v>31</v>
       </c>
       <c r="U61" s="11" t="s">
         <v>32</v>
@@ -5219,7 +5221,7 @@
         <v>0</v>
       </c>
       <c r="T63" s="12" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="U63" s="11" t="s">
         <v>32</v>
@@ -5478,7 +5480,7 @@
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46223.80773180556</v>
+        <v>46246.87418032407</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>244</v>
@@ -5904,7 +5906,7 @@
         <v>46241.20193481482</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
@@ -5997,7 +5999,7 @@
         <v>260</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="P76" s="6" t="s">
         <v>275</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-15 09:43 Chile
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -833,22 +833,22 @@
     <t>PACKING LIST,Logistica:</t>
   </si>
   <si>
+    <t>1213459189207091</t>
+  </si>
+  <si>
+    <t>PACKING LIST</t>
+  </si>
+  <si>
+    <t>Nicolás Mol</t>
+  </si>
+  <si>
+    <t>nicolas.mol@zitron.com</t>
+  </si>
+  <si>
+    <t>Despacho,Logistica:</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213459189207091</t>
-  </si>
-  <si>
-    <t>PACKING LIST</t>
-  </si>
-  <si>
-    <t>Nicolás Mol</t>
-  </si>
-  <si>
-    <t>nicolas.mol@zitron.com</t>
-  </si>
-  <si>
-    <t>Despacho,Logistica:</t>
   </si>
   <si>
     <t>1213459189153337</t>
@@ -5903,7 +5903,7 @@
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46248.25032157407</v>
+        <v>46249.19508818287</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>60</v>
@@ -5953,13 +5953,13 @@
       <c r="T75" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U75" s="12" t="s">
-        <v>270</v>
+      <c r="U75" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B76" s="5">
         <v>46079.83530269676</v>
@@ -5969,16 +5969,16 @@
         <v>46244.19896359954</v>
       </c>
       <c r="E76" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G76" s="6" t="s">
         <v>272</v>
       </c>
-      <c r="F76" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G76" s="6" t="s">
+      <c r="H76" s="6" t="s">
         <v>273</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>274</v>
       </c>
       <c r="I76" s="5">
         <v>46251</v>
@@ -6002,7 +6002,7 @@
         <v>60</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="Q76" s="5">
         <v>46251</v>
@@ -6017,7 +6017,7 @@
         <v>116</v>
       </c>
       <c r="U76" s="12" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -6038,10 +6038,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="H77" s="9" t="s">
         <v>273</v>
-      </c>
-      <c r="H77" s="9" t="s">
-        <v>274</v>
       </c>
       <c r="I77" s="8">
         <v>46252</v>
@@ -6062,7 +6062,7 @@
         <v>260</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="P77" s="9" t="s">
         <v>278</v>
@@ -6080,7 +6080,7 @@
         <v>116</v>
       </c>
       <c r="U77" s="12" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-08-19 13:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001518 - EQ CHAPARRAL B.xlsx
+++ b/data/50001518 - EQ CHAPARRAL B.xlsx
@@ -857,28 +857,28 @@
     <t>Gestion,Costos,Logistica:</t>
   </si>
   <si>
+    <t>1213459189153338</t>
+  </si>
+  <si>
+    <t>Cierre proyecto:</t>
+  </si>
+  <si>
+    <t>Gestion,Costos</t>
+  </si>
+  <si>
+    <t>1213459189153339</t>
+  </si>
+  <si>
+    <t>Gestion</t>
+  </si>
+  <si>
+    <t>Nicolás</t>
+  </si>
+  <si>
+    <t>nicolas.tello@zitron.com</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213459189153338</t>
-  </si>
-  <si>
-    <t>Cierre proyecto:</t>
-  </si>
-  <si>
-    <t>Gestion,Costos</t>
-  </si>
-  <si>
-    <t>1213459189153339</t>
-  </si>
-  <si>
-    <t>Gestion</t>
-  </si>
-  <si>
-    <t>Nicolás</t>
-  </si>
-  <si>
-    <t>nicolas.tello@zitron.com</t>
   </si>
   <si>
     <t>1213459189153340</t>
@@ -6029,7 +6029,7 @@
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46252.25019825231</v>
+        <v>46253.19238331019</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>276</v>
@@ -6079,13 +6079,13 @@
       <c r="T77" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U77" s="12" t="s">
-        <v>278</v>
+      <c r="U77" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B78" s="5">
         <v>46079.83530333333</v>
@@ -6095,7 +6095,7 @@
         <v>46090.67667782407</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>25</v>
@@ -6119,7 +6119,7 @@
         <v>26</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>26</v>
@@ -6132,26 +6132,26 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B79" s="8">
         <v>46079.83530363426</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46090.805033425924</v>
+        <v>46253.19261353009</v>
       </c>
       <c r="E79" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="F79" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="G79" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="F79" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="G79" s="9" t="s">
+      <c r="H79" s="9" t="s">
         <v>284</v>
-      </c>
-      <c r="H79" s="9" t="s">
-        <v>285</v>
       </c>
       <c r="I79" s="8">
         <v>46253</v>
@@ -6169,13 +6169,13 @@
         <v>26</v>
       </c>
       <c r="N79" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="O79" s="9" t="s">
         <v>276</v>
       </c>
       <c r="P79" s="9" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="Q79" s="8">
         <v>46252</v>
@@ -6189,8 +6189,8 @@
       <c r="T79" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U79" s="10" t="s">
-        <v>117</v>
+      <c r="U79" s="12" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
@@ -6202,7 +6202,7 @@
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46114.51489402778</v>
+        <v>46253.192614178246</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>287</v>
@@ -6211,10 +6211,10 @@
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="H80" s="6" t="s">
         <v>284</v>
-      </c>
-      <c r="H80" s="6" t="s">
-        <v>285</v>
       </c>
       <c r="I80" s="5">
         <v>46253</v>
@@ -6232,13 +6232,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="O80" s="6" t="s">
         <v>288</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="Q80" s="5">
         <v>46252</v>
@@ -6252,8 +6252,8 @@
       <c r="T80" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="U80" s="10" t="s">
-        <v>117</v>
+      <c r="U80" s="12" t="s">
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>